<commit_message>
Updated IQAC module, fixed template issue, added converter
</commit_message>
<xml_diff>
--- a/bridge.xlsx
+++ b/bridge.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,6 +443,556 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1a</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CO4</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1b</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CO4</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1c</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CO4</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CO5</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1e</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CO5</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1f</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CO5</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1g</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CO5</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CO6</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1i</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CO6</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1j</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CO6</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2a</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CO4</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2b</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CO4</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>3a</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CO5</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>3b</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CO5</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>4a</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CO5</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>4b</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CO5</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>5a</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CO5</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>5b</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CO5</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>L5</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>6a</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CO6</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>6b</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CO6</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CO6</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>7b</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CO6</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
my working version backup
</commit_message>
<xml_diff>
--- a/bridge.xlsx
+++ b/bridge.xlsx
@@ -459,12 +459,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -484,12 +484,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -534,12 +534,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -559,12 +559,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -609,12 +609,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -634,12 +634,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -654,17 +654,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CO6</t>
+          <t>CO3</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -684,12 +684,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>L4</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -734,7 +734,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>L4</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -750,7 +750,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -759,7 +759,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>L4</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -784,7 +784,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>L4</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -800,7 +800,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -809,7 +809,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>L4</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -834,7 +834,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>L4</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -850,16 +850,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CO5</t>
+          <t>CO6</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>L4</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -875,16 +875,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CO5</t>
+          <t>CO6</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>L5</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -900,7 +900,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -909,7 +909,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -925,16 +925,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CO6</t>
+          <t>CO3</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -950,16 +950,16 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CO6</t>
+          <t>CO4</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -984,7 +984,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">

</xml_diff>